<commit_message>
feat: add changes to Marg Analytics dashboard
</commit_message>
<xml_diff>
--- a/Marg-Analytics-Sales-Dashboard/Data & Analysis/MargAnalytics.xlsx
+++ b/Marg-Analytics-Sales-Dashboard/Data & Analysis/MargAnalytics.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/1561743a825db6f2/Documents/AkoladeDSJourney/Marg-Analytics-Sales-Dashboard/Data &amp; Analysis/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="2" documentId="13_ncr:1_{E5404A30-C17D-48AF-9C59-119882370D86}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{5E1EB2C7-49BE-4A1A-B631-4BCBA4DED640}"/>
+  <xr:revisionPtr revIDLastSave="326" documentId="13_ncr:1_{E5404A30-C17D-48AF-9C59-119882370D86}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{6B2D9D95-01D6-490C-9E99-6EA8215236E3}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" activeTab="1" xr2:uid="{FD736105-A461-4708-B902-2A05B2FF5345}"/>
   </bookViews>
@@ -21,13 +21,13 @@
   </definedNames>
   <calcPr calcId="191029"/>
   <pivotCaches>
-    <pivotCache cacheId="0" r:id="rId3"/>
-    <pivotCache cacheId="1" r:id="rId4"/>
-    <pivotCache cacheId="2" r:id="rId5"/>
-    <pivotCache cacheId="3" r:id="rId6"/>
-    <pivotCache cacheId="4" r:id="rId7"/>
-    <pivotCache cacheId="5" r:id="rId8"/>
-    <pivotCache cacheId="6" r:id="rId9"/>
+    <pivotCache cacheId="451" r:id="rId3"/>
+    <pivotCache cacheId="454" r:id="rId4"/>
+    <pivotCache cacheId="457" r:id="rId5"/>
+    <pivotCache cacheId="460" r:id="rId6"/>
+    <pivotCache cacheId="463" r:id="rId7"/>
+    <pivotCache cacheId="466" r:id="rId8"/>
+    <pivotCache cacheId="469" r:id="rId9"/>
   </pivotCaches>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{876F7934-8845-4945-9796-88D515C7AA90}">
@@ -324,7 +324,250 @@
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Percent" xfId="1" builtinId="5"/>
   </cellStyles>
-  <dxfs count="10">
+  <dxfs count="91">
+    <dxf>
+      <numFmt numFmtId="164" formatCode="[&gt;=1000000]\₦\ #,##0.00,,&quot;M&quot;;[&gt;=1000]\₦\ #.00,&quot;K&quot;;\₦\ ###.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="[&gt;=1000000]\₦\ #,##0.00,,&quot;M&quot;;[&gt;=1000]\₦\ #.00,&quot;K&quot;;\₦\ ###.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="[&gt;=1000000]\₦\ #,##0.00,,&quot;M&quot;;[&gt;=1000]\₦\ #.00,&quot;K&quot;;\₦\ ###.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="[&gt;=1000000]\₦\ #,##0.00,,&quot;M&quot;;[&gt;=1000]\₦\ #.00,&quot;K&quot;;\₦\ ###.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="1" formatCode="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="[&gt;=1000000]\₦\ #,##0.00,,&quot;M&quot;;[&gt;=1000]\₦\ #.00,&quot;K&quot;;\₦\ ###.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="[&gt;=1000000]\₦\ #,##0.00,,&quot;M&quot;;[&gt;=1000]\₦\ #.00,&quot;K&quot;;\₦\ ###.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="[&gt;=1000000]\₦\ #,##0.00,,&quot;M&quot;;[&gt;=1000]\₦\ #.00,&quot;K&quot;;\₦\ ###.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="[&gt;=1000000]\₦\ #,##0.00,,&quot;M&quot;;[&gt;=1000]\₦\ #.00,&quot;K&quot;;\₦\ ###.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="[&gt;=1000000]\₦\ #,##0.00,,&quot;M&quot;;[&gt;=1000]\₦\ #.00,&quot;K&quot;;\₦\ ###.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="[&gt;=1000000]\₦\ #,##0.00,,&quot;M&quot;;[&gt;=1000]\₦\ #.00,&quot;K&quot;;\₦\ ###.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="[&gt;=1000000]\₦\ #,##0.00,,&quot;M&quot;;[&gt;=1000]\₦\ #.00,&quot;K&quot;;\₦\ ###.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="[&gt;=1000000]\₦\ #,##0.00,,&quot;M&quot;;[&gt;=1000]\₦\ #.00,&quot;K&quot;;\₦\ ###.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="1" formatCode="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="[&gt;=1000000]\₦\ #,##0.00,,&quot;M&quot;;[&gt;=1000]\₦\ #.00,&quot;K&quot;;\₦\ ###.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="[&gt;=1000000]\₦\ #,##0.00,,&quot;M&quot;;[&gt;=1000]\₦\ #.00,&quot;K&quot;;\₦\ ###.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="[&gt;=1000000]\₦\ #,##0.00,,&quot;M&quot;;[&gt;=1000]\₦\ #.00,&quot;K&quot;;\₦\ ###.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="[&gt;=1000000]\₦\ #,##0.00,,&quot;M&quot;;[&gt;=1000]\₦\ #.00,&quot;K&quot;;\₦\ ###.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="[&gt;=1000000]\₦\ #,##0.00,,&quot;M&quot;;[&gt;=1000]\₦\ #.00,&quot;K&quot;;\₦\ ###.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="[&gt;=1000000]\₦\ #,##0.00,,&quot;M&quot;;[&gt;=1000]\₦\ #.00,&quot;K&quot;;\₦\ ###.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="[&gt;=1000000]\₦\ #,##0.00,,&quot;M&quot;;[&gt;=1000]\₦\ #.00,&quot;K&quot;;\₦\ ###.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="[&gt;=1000000]\₦\ #,##0.00,,&quot;M&quot;;[&gt;=1000]\₦\ #.00,&quot;K&quot;;\₦\ ###.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="1" formatCode="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="[&gt;=1000000]\₦\ #,##0.00,,&quot;M&quot;;[&gt;=1000]\₦\ #.00,&quot;K&quot;;\₦\ ###.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="[&gt;=1000000]\₦\ #,##0.00,,&quot;M&quot;;[&gt;=1000]\₦\ #.00,&quot;K&quot;;\₦\ ###.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="[&gt;=1000000]\₦\ #,##0.00,,&quot;M&quot;;[&gt;=1000]\₦\ #.00,&quot;K&quot;;\₦\ ###.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="[&gt;=1000000]\₦\ #,##0.00,,&quot;M&quot;;[&gt;=1000]\₦\ #.00,&quot;K&quot;;\₦\ ###.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="[&gt;=1000000]\₦\ #,##0.00,,&quot;M&quot;;[&gt;=1000]\₦\ #.00,&quot;K&quot;;\₦\ ###.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="[&gt;=1000000]\₦\ #,##0.00,,&quot;M&quot;;[&gt;=1000]\₦\ #.00,&quot;K&quot;;\₦\ ###.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="[&gt;=1000000]\₦\ #,##0.00,,&quot;M&quot;;[&gt;=1000]\₦\ #.00,&quot;K&quot;;\₦\ ###.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="[&gt;=1000000]\₦\ #,##0.00,,&quot;M&quot;;[&gt;=1000]\₦\ #.00,&quot;K&quot;;\₦\ ###.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="1" formatCode="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="[&gt;=1000000]\₦\ #,##0.00,,&quot;M&quot;;[&gt;=1000]\₦\ #.00,&quot;K&quot;;\₦\ ###.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="[&gt;=1000000]\₦\ #,##0.00,,&quot;M&quot;;[&gt;=1000]\₦\ #.00,&quot;K&quot;;\₦\ ###.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="[&gt;=1000000]\₦\ #,##0.00,,&quot;M&quot;;[&gt;=1000]\₦\ #.00,&quot;K&quot;;\₦\ ###.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="[&gt;=1000000]\₦\ #,##0.00,,&quot;M&quot;;[&gt;=1000]\₦\ #.00,&quot;K&quot;;\₦\ ###.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="[&gt;=1000000]\₦\ #,##0.00,,&quot;M&quot;;[&gt;=1000]\₦\ #.00,&quot;K&quot;;\₦\ ###.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="[&gt;=1000000]\₦\ #,##0.00,,&quot;M&quot;;[&gt;=1000]\₦\ #.00,&quot;K&quot;;\₦\ ###.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="[&gt;=1000000]\₦\ #,##0.00,,&quot;M&quot;;[&gt;=1000]\₦\ #.00,&quot;K&quot;;\₦\ ###.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="[&gt;=1000000]\₦\ #,##0.00,,&quot;M&quot;;[&gt;=1000]\₦\ #.00,&quot;K&quot;;\₦\ ###.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="1" formatCode="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="[&gt;=1000000]\₦\ #,##0.00,,&quot;M&quot;;[&gt;=1000]\₦\ #.00,&quot;K&quot;;\₦\ ###.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="[&gt;=1000000]\₦\ #,##0.00,,&quot;M&quot;;[&gt;=1000]\₦\ #.00,&quot;K&quot;;\₦\ ###.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="[&gt;=1000000]\₦\ #,##0.00,,&quot;M&quot;;[&gt;=1000]\₦\ #.00,&quot;K&quot;;\₦\ ###.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="[&gt;=1000000]\₦\ #,##0.00,,&quot;M&quot;;[&gt;=1000]\₦\ #.00,&quot;K&quot;;\₦\ ###.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="[&gt;=1000000]\₦\ #,##0.00,,&quot;M&quot;;[&gt;=1000]\₦\ #.00,&quot;K&quot;;\₦\ ###.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="[&gt;=1000000]\₦\ #,##0.00,,&quot;M&quot;;[&gt;=1000]\₦\ #.00,&quot;K&quot;;\₦\ ###.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="[&gt;=1000000]\₦\ #,##0.00,,&quot;M&quot;;[&gt;=1000]\₦\ #.00,&quot;K&quot;;\₦\ ###.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="[&gt;=1000000]\₦\ #,##0.00,,&quot;M&quot;;[&gt;=1000]\₦\ #.00,&quot;K&quot;;\₦\ ###.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="1" formatCode="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="[&gt;=1000000]\₦\ #,##0.00,,&quot;M&quot;;[&gt;=1000]\₦\ #.00,&quot;K&quot;;\₦\ ###.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="[&gt;=1000000]\₦\ #,##0.00,,&quot;M&quot;;[&gt;=1000]\₦\ #.00,&quot;K&quot;;\₦\ ###.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="[&gt;=1000000]\₦\ #,##0.00,,&quot;M&quot;;[&gt;=1000]\₦\ #.00,&quot;K&quot;;\₦\ ###.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="[&gt;=1000000]\₦\ #,##0.00,,&quot;M&quot;;[&gt;=1000]\₦\ #.00,&quot;K&quot;;\₦\ ###.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="[&gt;=1000000]\₦\ #,##0.00,,&quot;M&quot;;[&gt;=1000]\₦\ #.00,&quot;K&quot;;\₦\ ###.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="[&gt;=1000000]\₦\ #,##0.00,,&quot;M&quot;;[&gt;=1000]\₦\ #.00,&quot;K&quot;;\₦\ ###.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="[&gt;=1000000]\₦\ #,##0.00,,&quot;M&quot;;[&gt;=1000]\₦\ #.00,&quot;K&quot;;\₦\ ###.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="[&gt;=1000000]\₦\ #,##0.00,,&quot;M&quot;;[&gt;=1000]\₦\ #.00,&quot;K&quot;;\₦\ ###.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="1" formatCode="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="[&gt;=1000000]\₦\ #,##0.00,,&quot;M&quot;;[&gt;=1000]\₦\ #.00,&quot;K&quot;;\₦\ ###.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="[&gt;=1000000]\₦\ #,##0.00,,&quot;M&quot;;[&gt;=1000]\₦\ #.00,&quot;K&quot;;\₦\ ###.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="[&gt;=1000000]\₦\ #,##0.00,,&quot;M&quot;;[&gt;=1000]\₦\ #.00,&quot;K&quot;;\₦\ ###.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="[&gt;=1000000]\₦\ #,##0.00,,&quot;M&quot;;[&gt;=1000]\₦\ #.00,&quot;K&quot;;\₦\ ###.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="[&gt;=1000000]\₦\ #,##0.00,,&quot;M&quot;;[&gt;=1000]\₦\ #.00,&quot;K&quot;;\₦\ ###.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="[&gt;=1000000]\₦\ #,##0.00,,&quot;M&quot;;[&gt;=1000]\₦\ #.00,&quot;K&quot;;\₦\ ###.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="[&gt;=1000000]\₦\ #,##0.00,,&quot;M&quot;;[&gt;=1000]\₦\ #.00,&quot;K&quot;;\₦\ ###.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="[&gt;=1000000]\₦\ #,##0.00,,&quot;M&quot;;[&gt;=1000]\₦\ #.00,&quot;K&quot;;\₦\ ###.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="1" formatCode="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="[&gt;=1000000]\₦\ #,##0.00,,&quot;M&quot;;[&gt;=1000]\₦\ #.00,&quot;K&quot;;\₦\ ###.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="[&gt;=1000000]\₦\ #,##0.00,,&quot;M&quot;;[&gt;=1000]\₦\ #.00,&quot;K&quot;;\₦\ ###.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="[&gt;=1000000]\₦\ #,##0.00,,&quot;M&quot;;[&gt;=1000]\₦\ #.00,&quot;K&quot;;\₦\ ###.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="[&gt;=1000000]\₦\ #,##0.00,,&quot;M&quot;;[&gt;=1000]\₦\ #.00,&quot;K&quot;;\₦\ ###.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="[&gt;=1000000]\₦\ #,##0.00,,&quot;M&quot;;[&gt;=1000]\₦\ #.00,&quot;K&quot;;\₦\ ###.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="[&gt;=1000000]\₦\ #,##0.00,,&quot;M&quot;;[&gt;=1000]\₦\ #.00,&quot;K&quot;;\₦\ ###.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="[&gt;=1000000]\₦\ #,##0.00,,&quot;M&quot;;[&gt;=1000]\₦\ #.00,&quot;K&quot;;\₦\ ###.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="[&gt;=1000000]\₦\ #,##0.00,,&quot;M&quot;;[&gt;=1000]\₦\ #.00,&quot;K&quot;;\₦\ ###.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="1" formatCode="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="[&gt;=1000000]\₦\ #,##0.00,,&quot;M&quot;;[&gt;=1000]\₦\ #.00,&quot;K&quot;;\₦\ ###.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="[&gt;=1000000]\₦\ #,##0.00,,&quot;M&quot;;[&gt;=1000]\₦\ #.00,&quot;K&quot;;\₦\ ###.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="[&gt;=1000000]\₦\ #,##0.00,,&quot;M&quot;;[&gt;=1000]\₦\ #.00,&quot;K&quot;;\₦\ ###.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="[&gt;=1000000]\₦\ #,##0.00,,&quot;M&quot;;[&gt;=1000]\₦\ #.00,&quot;K&quot;;\₦\ ###.00"/>
+    </dxf>
     <dxf>
       <numFmt numFmtId="164" formatCode="[&gt;=1000000]\₦\ #,##0.00,,&quot;M&quot;;[&gt;=1000]\₦\ #.00,&quot;K&quot;;\₦\ ###.00"/>
     </dxf>
@@ -370,15 +613,15 @@
   </dxfs>
   <tableStyles count="1" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16">
     <tableStyle name="Slicer Style 1" pivot="0" table="0" count="5" xr9:uid="{F27145E4-A4F3-4C2E-9820-8D65AA9904DD}">
-      <tableStyleElement type="wholeTable" dxfId="9"/>
+      <tableStyleElement type="wholeTable" dxfId="90"/>
     </tableStyle>
   </tableStyles>
   <colors>
     <mruColors>
       <color rgb="FF2A1713"/>
+      <color rgb="FF956959"/>
       <color rgb="FFE9B48A"/>
       <color rgb="FF5C352C"/>
-      <color rgb="FF956959"/>
     </mruColors>
   </colors>
   <extLst>
@@ -478,6 +721,375 @@
 </file>
 
 <file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+  <c:date1904 val="0"/>
+  <c:lang val="en-US"/>
+  <c:roundedCorners val="0"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
+      <c14:style val="102"/>
+    </mc:Choice>
+    <mc:Fallback>
+      <c:style val="2"/>
+    </mc:Fallback>
+  </mc:AlternateContent>
+  <c:pivotSource>
+    <c:name>[MargAnalytics.xlsx]PivotTables!PivotTable7</c:name>
+    <c:fmtId val="10"/>
+  </c:pivotSource>
+  <c:chart>
+    <c:autoTitleDeleted val="1"/>
+    <c:pivotFmts>
+      <c:pivotFmt>
+        <c:idx val="0"/>
+        <c:spPr>
+          <a:solidFill>
+            <a:schemeClr val="accent1"/>
+          </a:solidFill>
+          <a:ln>
+            <a:noFill/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:marker>
+          <c:symbol val="none"/>
+        </c:marker>
+        <c:dLbl>
+          <c:idx val="0"/>
+          <c:delete val="1"/>
+          <c:extLst>
+            <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}"/>
+          </c:extLst>
+        </c:dLbl>
+      </c:pivotFmt>
+      <c:pivotFmt>
+        <c:idx val="1"/>
+        <c:spPr>
+          <a:solidFill>
+            <a:schemeClr val="accent1"/>
+          </a:solidFill>
+          <a:ln>
+            <a:noFill/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:marker>
+          <c:symbol val="none"/>
+        </c:marker>
+        <c:dLbl>
+          <c:idx val="0"/>
+          <c:delete val="1"/>
+          <c:extLst>
+            <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}"/>
+          </c:extLst>
+        </c:dLbl>
+      </c:pivotFmt>
+      <c:pivotFmt>
+        <c:idx val="2"/>
+        <c:spPr>
+          <a:solidFill>
+            <a:srgbClr val="956959">
+              <a:alpha val="82000"/>
+            </a:srgbClr>
+          </a:solidFill>
+          <a:ln>
+            <a:noFill/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:marker>
+          <c:symbol val="none"/>
+        </c:marker>
+        <c:dLbl>
+          <c:idx val="0"/>
+          <c:delete val="1"/>
+          <c:extLst>
+            <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}"/>
+          </c:extLst>
+        </c:dLbl>
+      </c:pivotFmt>
+      <c:pivotFmt>
+        <c:idx val="3"/>
+        <c:spPr>
+          <a:solidFill>
+            <a:srgbClr val="956959">
+              <a:alpha val="82000"/>
+            </a:srgbClr>
+          </a:solidFill>
+          <a:ln>
+            <a:noFill/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:marker>
+          <c:symbol val="none"/>
+        </c:marker>
+        <c:dLbl>
+          <c:idx val="0"/>
+          <c:delete val="1"/>
+          <c:extLst>
+            <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}"/>
+          </c:extLst>
+        </c:dLbl>
+      </c:pivotFmt>
+      <c:pivotFmt>
+        <c:idx val="4"/>
+        <c:spPr>
+          <a:solidFill>
+            <a:srgbClr val="956959">
+              <a:alpha val="82000"/>
+            </a:srgbClr>
+          </a:solidFill>
+          <a:ln>
+            <a:noFill/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:marker>
+          <c:symbol val="none"/>
+        </c:marker>
+        <c:dLbl>
+          <c:idx val="0"/>
+          <c:delete val="1"/>
+          <c:extLst>
+            <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}"/>
+          </c:extLst>
+        </c:dLbl>
+      </c:pivotFmt>
+      <c:pivotFmt>
+        <c:idx val="5"/>
+        <c:spPr>
+          <a:solidFill>
+            <a:srgbClr val="956959">
+              <a:alpha val="82000"/>
+            </a:srgbClr>
+          </a:solidFill>
+          <a:ln>
+            <a:noFill/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:marker>
+          <c:symbol val="none"/>
+        </c:marker>
+        <c:dLbl>
+          <c:idx val="0"/>
+          <c:delete val="1"/>
+          <c:extLst>
+            <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}"/>
+          </c:extLst>
+        </c:dLbl>
+      </c:pivotFmt>
+    </c:pivotFmts>
+    <c:plotArea>
+      <c:layout>
+        <c:manualLayout>
+          <c:layoutTarget val="inner"/>
+          <c:xMode val="edge"/>
+          <c:yMode val="edge"/>
+          <c:x val="0.11008961155288881"/>
+          <c:y val="0"/>
+          <c:w val="0.80318497164843272"/>
+          <c:h val="0.88251732956457363"/>
+        </c:manualLayout>
+      </c:layout>
+      <c:areaChart>
+        <c:grouping val="standard"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>PivotTables!$L$14</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>Total</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:solidFill>
+              <a:srgbClr val="956959">
+                <a:alpha val="82000"/>
+              </a:srgbClr>
+            </a:solidFill>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:cat>
+            <c:strRef>
+              <c:f>PivotTables!$K$15:$K$19</c:f>
+              <c:strCache>
+                <c:ptCount val="4"/>
+                <c:pt idx="0">
+                  <c:v>Corporate Sales</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>Marketplace</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>Online</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>Retail Store</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>PivotTables!$L$15:$L$19</c:f>
+              <c:numCache>
+                <c:formatCode>[&gt;=1000000]\₦\ #,##0.00,,"M";[&gt;=1000]\₦\ #.00,"K";\₦\ ###.00</c:formatCode>
+                <c:ptCount val="4"/>
+                <c:pt idx="0">
+                  <c:v>718745.00499999896</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>310402.93140000023</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>791536.99460000009</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>631399.37030000007</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000000-CECA-4A75-8FD2-FA73349F74DC}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:dLbls>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+        </c:dLbls>
+        <c:axId val="2007843152"/>
+        <c:axId val="2007846992"/>
+      </c:areaChart>
+      <c:catAx>
+        <c:axId val="2007843152"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="out"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:noFill/>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="b" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="800" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:srgbClr val="2A1713"/>
+                </a:solidFill>
+                <a:latin typeface="Franklin Gothic Medium" panose="020B0603020102020204" pitchFamily="34" charset="0"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="2007846992"/>
+        <c:crosses val="autoZero"/>
+        <c:auto val="1"/>
+        <c:lblAlgn val="ctr"/>
+        <c:lblOffset val="100"/>
+        <c:noMultiLvlLbl val="0"/>
+      </c:catAx>
+      <c:valAx>
+        <c:axId val="2007846992"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="1"/>
+        <c:axPos val="l"/>
+        <c:numFmt formatCode="[&gt;=1000000]\₦\ #,##0.00,,&quot;M&quot;;[&gt;=1000]\₦\ #.00,&quot;K&quot;;\₦\ ###.00" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:crossAx val="2007843152"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="midCat"/>
+      </c:valAx>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+      </c:spPr>
+    </c:plotArea>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="zero"/>
+    <c:showDLblsOverMax val="0"/>
+    <c:extLst/>
+  </c:chart>
+  <c:spPr>
+    <a:noFill/>
+    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+      <a:noFill/>
+      <a:round/>
+    </a:ln>
+    <a:effectLst/>
+  </c:spPr>
+  <c:txPr>
+    <a:bodyPr/>
+    <a:lstStyle/>
+    <a:p>
+      <a:pPr>
+        <a:defRPr/>
+      </a:pPr>
+      <a:endParaRPr lang="en-US"/>
+    </a:p>
+  </c:txPr>
+  <c:printSettings>
+    <c:headerFooter/>
+    <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
+    <c:pageSetup/>
+  </c:printSettings>
+  <c:extLst>
+    <c:ext xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" uri="{781A3756-C4B2-4CAC-9D66-4F8BD8637D16}">
+      <c14:pivotOptions>
+        <c14:dropZoneFilter val="1"/>
+        <c14:dropZoneCategories val="1"/>
+        <c14:dropZoneData val="1"/>
+      </c14:pivotOptions>
+    </c:ext>
+    <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{E28EC0CA-F0BB-4C9C-879D-F8772B89E7AC}">
+      <c16:pivotOptions16>
+        <c16:showExpandCollapseFieldButtons val="1"/>
+      </c16:pivotOptions16>
+    </c:ext>
+  </c:extLst>
+</c:chartSpace>
+</file>
+
+<file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
 <c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
   <c:date1904 val="0"/>
   <c:lang val="en-US"/>
@@ -965,7 +1577,7 @@
 </c:chartSpace>
 </file>
 
-<file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/charts/chart3.xml><?xml version="1.0" encoding="utf-8"?>
 <c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
   <c:date1904 val="0"/>
   <c:lang val="en-US"/>
@@ -1235,7 +1847,7 @@
             <a:effectLst/>
           </c:spPr>
           <c:txPr>
-            <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
+            <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="overflow" horzOverflow="overflow" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
               <a:spAutoFit/>
             </a:bodyPr>
             <a:lstStyle/>
@@ -1376,7 +1988,7 @@
               <a:effectLst/>
             </c:spPr>
             <c:txPr>
-              <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
+              <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="overflow" horzOverflow="overflow" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
                 <a:spAutoFit/>
               </a:bodyPr>
               <a:lstStyle/>
@@ -1698,7 +2310,7 @@
 </c:chartSpace>
 </file>
 
-<file path=xl/charts/chart3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/charts/chart4.xml><?xml version="1.0" encoding="utf-8"?>
 <c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
   <c:date1904 val="0"/>
   <c:lang val="en-US"/>
@@ -1878,7 +2490,17 @@
       </c:pivotFmt>
     </c:pivotFmts>
     <c:plotArea>
-      <c:layout/>
+      <c:layout>
+        <c:manualLayout>
+          <c:layoutTarget val="inner"/>
+          <c:xMode val="edge"/>
+          <c:yMode val="edge"/>
+          <c:x val="0.25969423572875766"/>
+          <c:y val="0"/>
+          <c:w val="0.73745487832608536"/>
+          <c:h val="1"/>
+        </c:manualLayout>
+      </c:layout>
       <c:barChart>
         <c:barDir val="bar"/>
         <c:grouping val="clustered"/>
@@ -2149,7 +2771,7 @@
 </c:chartSpace>
 </file>
 
-<file path=xl/charts/chart4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/charts/chart5.xml><?xml version="1.0" encoding="utf-8"?>
 <c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
   <c:date1904 val="0"/>
   <c:lang val="en-US"/>
@@ -2167,7 +2789,69 @@
     <c:fmtId val="6"/>
   </c:pivotSource>
   <c:chart>
-    <c:autoTitleDeleted val="1"/>
+    <c:title>
+      <c:tx>
+        <c:rich>
+          <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="1200" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+                <a:solidFill>
+                  <a:srgbClr val="2A1713"/>
+                </a:solidFill>
+                <a:latin typeface="Franklin Gothic Medium" panose="020B0603020102020204" pitchFamily="34" charset="0"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:r>
+              <a:rPr lang="en-US" sz="1200">
+                <a:solidFill>
+                  <a:srgbClr val="2A1713"/>
+                </a:solidFill>
+                <a:latin typeface="Franklin Gothic Medium" panose="020B0603020102020204" pitchFamily="34" charset="0"/>
+              </a:rPr>
+              <a:t>Revenue by Customer Type</a:t>
+            </a:r>
+          </a:p>
+        </c:rich>
+      </c:tx>
+      <c:layout>
+        <c:manualLayout>
+          <c:xMode val="edge"/>
+          <c:yMode val="edge"/>
+          <c:x val="1.3095266494323084E-3"/>
+          <c:y val="0"/>
+        </c:manualLayout>
+      </c:layout>
+      <c:overlay val="1"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="1200" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+              <a:solidFill>
+                <a:srgbClr val="2A1713"/>
+              </a:solidFill>
+              <a:latin typeface="Franklin Gothic Medium" panose="020B0603020102020204" pitchFamily="34" charset="0"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="en-US"/>
+        </a:p>
+      </c:txPr>
+    </c:title>
+    <c:autoTitleDeleted val="0"/>
     <c:pivotFmts>
       <c:pivotFmt>
         <c:idx val="0"/>
@@ -2512,6 +3196,37 @@
         <a:effectLst/>
       </c:spPr>
     </c:plotArea>
+    <c:legend>
+      <c:legendPos val="l"/>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="en-US"/>
+        </a:p>
+      </c:txPr>
+    </c:legend>
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>
     <c:extLst>
@@ -2525,7 +3240,7 @@
   </c:chart>
   <c:spPr>
     <a:noFill/>
-    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+    <a:ln w="3175" cap="flat" cmpd="sng" algn="ctr">
       <a:solidFill>
         <a:srgbClr val="5C352C"/>
       </a:solidFill>
@@ -2552,6 +3267,7 @@
     <c:ext xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" uri="{781A3756-C4B2-4CAC-9D66-4F8BD8637D16}">
       <c14:pivotOptions>
         <c14:dropZoneFilter val="1"/>
+        <c14:dropZoneCategories val="1"/>
         <c14:dropZoneData val="1"/>
         <c14:dropZoneSeries val="1"/>
       </c14:pivotOptions>
@@ -4775,15 +5491,15 @@
   <xdr:twoCellAnchor>
     <xdr:from>
       <xdr:col>0</xdr:col>
-      <xdr:colOff>133350</xdr:colOff>
+      <xdr:colOff>57150</xdr:colOff>
       <xdr:row>0</xdr:row>
-      <xdr:rowOff>11588</xdr:rowOff>
+      <xdr:rowOff>21113</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>20</xdr:col>
-      <xdr:colOff>130302</xdr:colOff>
+      <xdr:colOff>54102</xdr:colOff>
       <xdr:row>36</xdr:row>
-      <xdr:rowOff>11588</xdr:rowOff>
+      <xdr:rowOff>21113</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
@@ -4798,8 +5514,8 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="133350" y="11588"/>
-          <a:ext cx="12255213" cy="6858000"/>
+          <a:off x="57150" y="21113"/>
+          <a:ext cx="12188952" cy="6858000"/>
         </a:xfrm>
         <a:prstGeom prst="roundRect">
           <a:avLst>
@@ -4908,6 +5624,44 @@
         </a:p>
       </xdr:txBody>
     </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>244928</xdr:colOff>
+      <xdr:row>9</xdr:row>
+      <xdr:rowOff>91108</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>402335</xdr:colOff>
+      <xdr:row>18</xdr:row>
+      <xdr:rowOff>545</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="17" name="Chart 16">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{D6916D6E-3D00-4B07-A73D-6FE895187DE0}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvGraphicFramePr>
+          <a:graphicFrameLocks/>
+        </xdr:cNvGraphicFramePr>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
     <xdr:clientData/>
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor>
@@ -5465,7 +6219,7 @@
       </xdr:xfrm>
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId2"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -5503,7 +6257,7 @@
       </xdr:xfrm>
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId2"/>
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId3"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -5511,14 +6265,14 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>12</xdr:col>
-      <xdr:colOff>171449</xdr:colOff>
+      <xdr:col>13</xdr:col>
+      <xdr:colOff>134468</xdr:colOff>
       <xdr:row>22</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>19</xdr:col>
-      <xdr:colOff>340098</xdr:colOff>
+      <xdr:col>20</xdr:col>
+      <xdr:colOff>22409</xdr:colOff>
       <xdr:row>33</xdr:row>
       <xdr:rowOff>169214</xdr:rowOff>
     </xdr:to>
@@ -5541,7 +6295,7 @@
       </xdr:xfrm>
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId3"/>
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId4"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -5550,15 +6304,15 @@
   <xdr:twoCellAnchor>
     <xdr:from>
       <xdr:col>8</xdr:col>
-      <xdr:colOff>326573</xdr:colOff>
-      <xdr:row>22</xdr:row>
-      <xdr:rowOff>10406</xdr:rowOff>
+      <xdr:colOff>240848</xdr:colOff>
+      <xdr:row>21</xdr:row>
+      <xdr:rowOff>86606</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>11</xdr:col>
-      <xdr:colOff>236112</xdr:colOff>
-      <xdr:row>30</xdr:row>
-      <xdr:rowOff>123182</xdr:rowOff>
+      <xdr:col>12</xdr:col>
+      <xdr:colOff>180975</xdr:colOff>
+      <xdr:row>32</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
@@ -5579,7 +6333,7 @@
       </xdr:xfrm>
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId4"/>
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId5"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -5587,16 +6341,16 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>8</xdr:col>
-      <xdr:colOff>568780</xdr:colOff>
-      <xdr:row>31</xdr:row>
-      <xdr:rowOff>2712</xdr:rowOff>
+      <xdr:col>9</xdr:col>
+      <xdr:colOff>152400</xdr:colOff>
+      <xdr:row>32</xdr:row>
+      <xdr:rowOff>21762</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>11</xdr:col>
-      <xdr:colOff>76524</xdr:colOff>
-      <xdr:row>34</xdr:row>
-      <xdr:rowOff>76669</xdr:rowOff>
+      <xdr:col>12</xdr:col>
+      <xdr:colOff>171451</xdr:colOff>
+      <xdr:row>33</xdr:row>
+      <xdr:rowOff>123825</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
@@ -5613,8 +6367,8 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="5467351" y="5908212"/>
-          <a:ext cx="1344709" cy="645457"/>
+          <a:off x="5638800" y="6117762"/>
+          <a:ext cx="1847851" cy="292563"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -5790,21 +6544,14 @@
           </a:lvl9pPr>
         </a:lstStyle>
         <a:p>
-          <a:r>
-            <a:rPr lang="en-US">
-              <a:solidFill>
-                <a:srgbClr val="2A1713"/>
-              </a:solidFill>
-            </a:rPr>
-            <a:t>Returning Customers</a:t>
-          </a:r>
+          <a:pPr algn="ctr"/>
           <a:r>
             <a:rPr lang="en-US" baseline="0">
               <a:solidFill>
                 <a:srgbClr val="2A1713"/>
               </a:solidFill>
             </a:rPr>
-            <a:t> generate more revenue</a:t>
+            <a:t>Revenue comes from </a:t>
           </a:r>
           <a:endParaRPr lang="en-US">
             <a:solidFill>
@@ -5818,16 +6565,16 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>9</xdr:col>
-      <xdr:colOff>107498</xdr:colOff>
+      <xdr:col>10</xdr:col>
+      <xdr:colOff>97973</xdr:colOff>
       <xdr:row>25</xdr:row>
-      <xdr:rowOff>19049</xdr:rowOff>
+      <xdr:rowOff>123824</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>10</xdr:col>
-      <xdr:colOff>440873</xdr:colOff>
+      <xdr:col>11</xdr:col>
+      <xdr:colOff>431348</xdr:colOff>
       <xdr:row>27</xdr:row>
-      <xdr:rowOff>28575</xdr:rowOff>
+      <xdr:rowOff>133350</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="PivotTables!$F$21">
       <xdr:nvSpPr>
@@ -5842,7 +6589,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="5593898" y="4781549"/>
+          <a:off x="6193973" y="4886324"/>
           <a:ext cx="942975" cy="390526"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -5979,14 +6726,14 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>12</xdr:col>
-      <xdr:colOff>171449</xdr:colOff>
+      <xdr:col>13</xdr:col>
+      <xdr:colOff>134468</xdr:colOff>
       <xdr:row>20</xdr:row>
       <xdr:rowOff>152399</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>17</xdr:col>
-      <xdr:colOff>180974</xdr:colOff>
+      <xdr:col>18</xdr:col>
+      <xdr:colOff>143992</xdr:colOff>
       <xdr:row>22</xdr:row>
       <xdr:rowOff>28574</xdr:rowOff>
     </xdr:to>
@@ -6003,8 +6750,8 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="7486649" y="3962399"/>
-          <a:ext cx="3057525" cy="257175"/>
+          <a:off x="8000997" y="3962399"/>
+          <a:ext cx="3035113" cy="257175"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -6387,11 +7134,392 @@
     </xdr:sp>
     <xdr:clientData/>
   </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>8</xdr:col>
+      <xdr:colOff>342900</xdr:colOff>
+      <xdr:row>31</xdr:row>
+      <xdr:rowOff>161925</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>10</xdr:col>
+      <xdr:colOff>304800</xdr:colOff>
+      <xdr:row>34</xdr:row>
+      <xdr:rowOff>142875</xdr:rowOff>
+    </xdr:to>
+    <xdr:grpSp>
+      <xdr:nvGrpSpPr>
+        <xdr:cNvPr id="28" name="Group 27">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{95CABF77-3724-9849-7311-6263C3176721}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvGrpSpPr/>
+      </xdr:nvGrpSpPr>
+      <xdr:grpSpPr>
+        <a:xfrm>
+          <a:off x="5207977" y="6067425"/>
+          <a:ext cx="1178169" cy="552450"/>
+          <a:chOff x="5241471" y="6067425"/>
+          <a:chExt cx="1186543" cy="552450"/>
+        </a:xfrm>
+      </xdr:grpSpPr>
+      <xdr:sp macro="" textlink="PivotTables!$F$21">
+        <xdr:nvSpPr>
+          <xdr:cNvPr id="25" name="TextBox 24">
+            <a:extLst>
+              <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{DFF30B98-8D20-8E65-4E3D-CF0C88B77B7B}"/>
+              </a:ext>
+            </a:extLst>
+          </xdr:cNvPr>
+          <xdr:cNvSpPr txBox="1"/>
+        </xdr:nvSpPr>
+        <xdr:spPr>
+          <a:xfrm>
+            <a:off x="5241471" y="6067425"/>
+            <a:ext cx="862695" cy="342900"/>
+          </a:xfrm>
+          <a:prstGeom prst="rect">
+            <a:avLst/>
+          </a:prstGeom>
+          <a:noFill/>
+          <a:ln w="9525" cmpd="sng">
+            <a:noFill/>
+          </a:ln>
+        </xdr:spPr>
+        <xdr:style>
+          <a:lnRef idx="0">
+            <a:scrgbClr r="0" g="0" b="0"/>
+          </a:lnRef>
+          <a:fillRef idx="0">
+            <a:scrgbClr r="0" g="0" b="0"/>
+          </a:fillRef>
+          <a:effectRef idx="0">
+            <a:scrgbClr r="0" g="0" b="0"/>
+          </a:effectRef>
+          <a:fontRef idx="minor">
+            <a:schemeClr val="dk1"/>
+          </a:fontRef>
+        </xdr:style>
+        <xdr:txBody>
+          <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="square" rtlCol="0" anchor="ctr"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr algn="l"/>
+            <a:fld id="{5D13EC03-9D2E-4DF4-8D59-5F650C38DA8F}" type="TxLink">
+              <a:rPr lang="en-US" sz="1200" b="0" i="0" u="none" strike="noStrike">
+                <a:solidFill>
+                  <a:srgbClr val="2A1713"/>
+                </a:solidFill>
+                <a:latin typeface="Franklin Gothic Medium" panose="020B0603020102020204" pitchFamily="34" charset="0"/>
+              </a:rPr>
+              <a:t>68.65%</a:t>
+            </a:fld>
+            <a:endParaRPr lang="en-US" sz="2000" b="0">
+              <a:solidFill>
+                <a:srgbClr val="2A1713"/>
+              </a:solidFill>
+              <a:latin typeface="Franklin Gothic Medium" panose="020B0603020102020204" pitchFamily="34" charset="0"/>
+            </a:endParaRPr>
+          </a:p>
+        </xdr:txBody>
+      </xdr:sp>
+      <xdr:sp macro="" textlink="PivotTables!$E$21">
+        <xdr:nvSpPr>
+          <xdr:cNvPr id="26" name="TextBox 25">
+            <a:extLst>
+              <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{047948DF-D037-5AD1-015A-C3254D592860}"/>
+              </a:ext>
+            </a:extLst>
+          </xdr:cNvPr>
+          <xdr:cNvSpPr txBox="1"/>
+        </xdr:nvSpPr>
+        <xdr:spPr>
+          <a:xfrm>
+            <a:off x="5422447" y="6276975"/>
+            <a:ext cx="1005567" cy="342900"/>
+          </a:xfrm>
+          <a:prstGeom prst="rect">
+            <a:avLst/>
+          </a:prstGeom>
+          <a:noFill/>
+          <a:ln w="9525" cmpd="sng">
+            <a:noFill/>
+          </a:ln>
+        </xdr:spPr>
+        <xdr:style>
+          <a:lnRef idx="0">
+            <a:scrgbClr r="0" g="0" b="0"/>
+          </a:lnRef>
+          <a:fillRef idx="0">
+            <a:scrgbClr r="0" g="0" b="0"/>
+          </a:fillRef>
+          <a:effectRef idx="0">
+            <a:scrgbClr r="0" g="0" b="0"/>
+          </a:effectRef>
+          <a:fontRef idx="minor">
+            <a:schemeClr val="dk1"/>
+          </a:fontRef>
+        </xdr:style>
+        <xdr:txBody>
+          <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="square" rtlCol="0" anchor="ctr"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr algn="l"/>
+            <a:fld id="{F75F2EEA-AC56-48F1-90BC-F0A3A25A213C}" type="TxLink">
+              <a:rPr lang="en-US" sz="1200" b="0" i="0" u="none" strike="noStrike">
+                <a:solidFill>
+                  <a:srgbClr val="2A1713"/>
+                </a:solidFill>
+                <a:latin typeface="Franklin Gothic Medium" panose="020B0603020102020204" pitchFamily="34" charset="0"/>
+              </a:rPr>
+              <a:t>Returning</a:t>
+            </a:fld>
+            <a:endParaRPr lang="en-US" sz="2400" b="0">
+              <a:solidFill>
+                <a:srgbClr val="2A1713"/>
+              </a:solidFill>
+              <a:latin typeface="Franklin Gothic Medium" panose="020B0603020102020204" pitchFamily="34" charset="0"/>
+            </a:endParaRPr>
+          </a:p>
+        </xdr:txBody>
+      </xdr:sp>
+    </xdr:grpSp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>10</xdr:col>
+      <xdr:colOff>152401</xdr:colOff>
+      <xdr:row>33</xdr:row>
+      <xdr:rowOff>50337</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>12</xdr:col>
+      <xdr:colOff>114301</xdr:colOff>
+      <xdr:row>34</xdr:row>
+      <xdr:rowOff>152400</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="27" name="Text Placeholder 387">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{43231612-A4EC-0A30-FEE9-0ABF95ECAB31}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr>
+          <a:spLocks noGrp="1"/>
+        </xdr:cNvSpPr>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="6275615" y="6336837"/>
+          <a:ext cx="1186543" cy="292563"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+      </xdr:spPr>
+      <xdr:txBody>
+        <a:bodyPr vert="horz" wrap="square" lIns="0" tIns="45720" rIns="0" bIns="45720" rtlCol="0" anchor="t">
+          <a:noAutofit/>
+        </a:bodyPr>
+        <a:lstStyle>
+          <a:lvl1pPr marL="0" indent="0" algn="ctr" defTabSz="914400" rtl="0" eaLnBrk="1" latinLnBrk="0" hangingPunct="1">
+            <a:lnSpc>
+              <a:spcPct val="90000"/>
+            </a:lnSpc>
+            <a:spcBef>
+              <a:spcPts val="1000"/>
+            </a:spcBef>
+            <a:buFont typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
+            <a:buNone/>
+            <a:defRPr sz="1200" kern="1200">
+              <a:solidFill>
+                <a:schemeClr val="bg1"/>
+              </a:solidFill>
+              <a:latin typeface="+mj-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:lvl1pPr>
+          <a:lvl2pPr marL="685800" indent="-228600" algn="l" defTabSz="914400" rtl="0" eaLnBrk="1" latinLnBrk="0" hangingPunct="1">
+            <a:lnSpc>
+              <a:spcPct val="90000"/>
+            </a:lnSpc>
+            <a:spcBef>
+              <a:spcPts val="500"/>
+            </a:spcBef>
+            <a:buFont typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
+            <a:buChar char="•"/>
+            <a:defRPr sz="2400" kern="1200">
+              <a:solidFill>
+                <a:schemeClr val="bg1"/>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:lvl2pPr>
+          <a:lvl3pPr marL="1143000" indent="-228600" algn="l" defTabSz="914400" rtl="0" eaLnBrk="1" latinLnBrk="0" hangingPunct="1">
+            <a:lnSpc>
+              <a:spcPct val="90000"/>
+            </a:lnSpc>
+            <a:spcBef>
+              <a:spcPts val="500"/>
+            </a:spcBef>
+            <a:buFont typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
+            <a:buChar char="•"/>
+            <a:defRPr sz="2000" kern="1200">
+              <a:solidFill>
+                <a:schemeClr val="bg1"/>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:lvl3pPr>
+          <a:lvl4pPr marL="1600200" indent="-228600" algn="l" defTabSz="914400" rtl="0" eaLnBrk="1" latinLnBrk="0" hangingPunct="1">
+            <a:lnSpc>
+              <a:spcPct val="90000"/>
+            </a:lnSpc>
+            <a:spcBef>
+              <a:spcPts val="500"/>
+            </a:spcBef>
+            <a:buFont typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
+            <a:buChar char="•"/>
+            <a:defRPr sz="1800" kern="1200">
+              <a:solidFill>
+                <a:schemeClr val="bg1"/>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:lvl4pPr>
+          <a:lvl5pPr marL="2057400" indent="-228600" algn="l" defTabSz="914400" rtl="0" eaLnBrk="1" latinLnBrk="0" hangingPunct="1">
+            <a:lnSpc>
+              <a:spcPct val="90000"/>
+            </a:lnSpc>
+            <a:spcBef>
+              <a:spcPts val="500"/>
+            </a:spcBef>
+            <a:buFont typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
+            <a:buChar char="•"/>
+            <a:defRPr sz="1800" kern="1200">
+              <a:solidFill>
+                <a:schemeClr val="bg1"/>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:lvl5pPr>
+          <a:lvl6pPr marL="2514600" indent="-228600" algn="l" defTabSz="914400" rtl="0" eaLnBrk="1" latinLnBrk="0" hangingPunct="1">
+            <a:lnSpc>
+              <a:spcPct val="90000"/>
+            </a:lnSpc>
+            <a:spcBef>
+              <a:spcPts val="500"/>
+            </a:spcBef>
+            <a:buFont typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
+            <a:buChar char="•"/>
+            <a:defRPr sz="1800" kern="1200">
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:lvl6pPr>
+          <a:lvl7pPr marL="2971800" indent="-228600" algn="l" defTabSz="914400" rtl="0" eaLnBrk="1" latinLnBrk="0" hangingPunct="1">
+            <a:lnSpc>
+              <a:spcPct val="90000"/>
+            </a:lnSpc>
+            <a:spcBef>
+              <a:spcPts val="500"/>
+            </a:spcBef>
+            <a:buFont typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
+            <a:buChar char="•"/>
+            <a:defRPr sz="1800" kern="1200">
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:lvl7pPr>
+          <a:lvl8pPr marL="3429000" indent="-228600" algn="l" defTabSz="914400" rtl="0" eaLnBrk="1" latinLnBrk="0" hangingPunct="1">
+            <a:lnSpc>
+              <a:spcPct val="90000"/>
+            </a:lnSpc>
+            <a:spcBef>
+              <a:spcPts val="500"/>
+            </a:spcBef>
+            <a:buFont typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
+            <a:buChar char="•"/>
+            <a:defRPr sz="1800" kern="1200">
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:lvl8pPr>
+          <a:lvl9pPr marL="3886200" indent="-228600" algn="l" defTabSz="914400" rtl="0" eaLnBrk="1" latinLnBrk="0" hangingPunct="1">
+            <a:lnSpc>
+              <a:spcPct val="90000"/>
+            </a:lnSpc>
+            <a:spcBef>
+              <a:spcPts val="500"/>
+            </a:spcBef>
+            <a:buFont typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
+            <a:buChar char="•"/>
+            <a:defRPr sz="1800" kern="1200">
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:lvl9pPr>
+        </a:lstStyle>
+        <a:p>
+          <a:pPr algn="l"/>
+          <a:r>
+            <a:rPr lang="en-US" baseline="0">
+              <a:solidFill>
+                <a:srgbClr val="2A1713"/>
+              </a:solidFill>
+            </a:rPr>
+            <a:t>customers</a:t>
+          </a:r>
+          <a:endParaRPr lang="en-US">
+            <a:solidFill>
+              <a:srgbClr val="2A1713"/>
+            </a:solidFill>
+          </a:endParaRPr>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
 </xdr:wsDr>
 </file>
 
 <file path=xl/pivotCache/pivotCacheDefinition1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" saveData="0" refreshedBy="KOLADE" refreshedDate="46293.974186226849" backgroundQuery="1" createdVersion="8" refreshedVersion="8" minRefreshableVersion="3" recordCount="0" supportSubquery="1" supportAdvancedDrill="1" xr:uid="{A7FE0B55-00E4-4068-B4D9-80A2148B07D3}">
+<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" saveData="0" refreshedBy="KOLADE" refreshedDate="46294.664676273147" backgroundQuery="1" createdVersion="8" refreshedVersion="8" minRefreshableVersion="3" recordCount="0" supportSubquery="1" supportAdvancedDrill="1" xr:uid="{A7FE0B55-00E4-4068-B4D9-80A2148B07D3}">
   <cacheSource type="external" connectionId="2"/>
   <cacheFields count="5">
     <cacheField name="[Measures].[Total Revenue]" caption="Total Revenue" numFmtId="0" hierarchy="14" level="32767"/>
@@ -6465,7 +7593,7 @@
 </file>
 
 <file path=xl/pivotCache/pivotCacheDefinition2.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" saveData="0" refreshedBy="KOLADE" refreshedDate="46293.97418784722" backgroundQuery="1" createdVersion="8" refreshedVersion="8" minRefreshableVersion="3" recordCount="0" supportSubquery="1" supportAdvancedDrill="1" xr:uid="{8464195A-B64C-4F10-B4E8-5AB7970649FA}">
+<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" saveData="0" refreshedBy="KOLADE" refreshedDate="46294.664677199071" backgroundQuery="1" createdVersion="8" refreshedVersion="8" minRefreshableVersion="3" recordCount="0" supportSubquery="1" supportAdvancedDrill="1" xr:uid="{8464195A-B64C-4F10-B4E8-5AB7970649FA}">
   <cacheSource type="external" connectionId="2"/>
   <cacheFields count="3">
     <cacheField name="[Measures].[Total Revenue]" caption="Total Revenue" numFmtId="0" hierarchy="14" level="32767"/>
@@ -6545,7 +7673,7 @@
 </file>
 
 <file path=xl/pivotCache/pivotCacheDefinition3.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" saveData="0" refreshedBy="KOLADE" refreshedDate="46293.974189120374" backgroundQuery="1" createdVersion="8" refreshedVersion="8" minRefreshableVersion="3" recordCount="0" supportSubquery="1" supportAdvancedDrill="1" xr:uid="{4C294FB0-2581-446B-B2B0-32084E9C7D8D}">
+<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" saveData="0" refreshedBy="KOLADE" refreshedDate="46294.664678009256" backgroundQuery="1" createdVersion="8" refreshedVersion="8" minRefreshableVersion="3" recordCount="0" supportSubquery="1" supportAdvancedDrill="1" xr:uid="{4C294FB0-2581-446B-B2B0-32084E9C7D8D}">
   <cacheSource type="external" connectionId="2"/>
   <cacheFields count="2">
     <cacheField name="[Measures].[Total Revenue]" caption="Total Revenue" numFmtId="0" hierarchy="14" level="32767"/>
@@ -6610,7 +7738,7 @@
 </file>
 
 <file path=xl/pivotCache/pivotCacheDefinition4.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" saveData="0" refreshedBy="KOLADE" refreshedDate="46293.974190393521" backgroundQuery="1" createdVersion="8" refreshedVersion="8" minRefreshableVersion="3" recordCount="0" supportSubquery="1" supportAdvancedDrill="1" xr:uid="{9A9A6D95-53C5-4373-B393-5A87F9E835A7}">
+<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" saveData="0" refreshedBy="KOLADE" refreshedDate="46294.664678935187" backgroundQuery="1" createdVersion="8" refreshedVersion="8" minRefreshableVersion="3" recordCount="0" supportSubquery="1" supportAdvancedDrill="1" xr:uid="{9A9A6D95-53C5-4373-B393-5A87F9E835A7}">
   <cacheSource type="external" connectionId="2"/>
   <cacheFields count="4">
     <cacheField name="[Measures].[Total Revenue]" caption="Total Revenue" numFmtId="0" hierarchy="14" level="32767"/>
@@ -6689,7 +7817,7 @@
 </file>
 
 <file path=xl/pivotCache/pivotCacheDefinition5.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" saveData="0" refreshedBy="KOLADE" refreshedDate="46293.974191898145" backgroundQuery="1" createdVersion="8" refreshedVersion="8" minRefreshableVersion="3" recordCount="0" supportSubquery="1" supportAdvancedDrill="1" xr:uid="{56979DD0-2DD3-43D5-9669-2B2DA8965249}">
+<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" saveData="0" refreshedBy="KOLADE" refreshedDate="46294.664679629626" backgroundQuery="1" createdVersion="8" refreshedVersion="8" minRefreshableVersion="3" recordCount="0" supportSubquery="1" supportAdvancedDrill="1" xr:uid="{56979DD0-2DD3-43D5-9669-2B2DA8965249}">
   <cacheSource type="external" connectionId="2"/>
   <cacheFields count="3">
     <cacheField name="[Measures].[Total Revenue]" caption="Total Revenue" numFmtId="0" hierarchy="14" level="32767"/>
@@ -6759,7 +7887,7 @@
 </file>
 
 <file path=xl/pivotCache/pivotCacheDefinition6.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" saveData="0" refreshedBy="KOLADE" refreshedDate="46293.97419375" backgroundQuery="1" createdVersion="8" refreshedVersion="8" minRefreshableVersion="3" recordCount="0" supportSubquery="1" supportAdvancedDrill="1" xr:uid="{36D1781F-D43F-4D67-BDF8-463496026D57}">
+<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" saveData="0" refreshedBy="KOLADE" refreshedDate="46294.664680439811" backgroundQuery="1" createdVersion="8" refreshedVersion="8" minRefreshableVersion="3" recordCount="0" supportSubquery="1" supportAdvancedDrill="1" xr:uid="{36D1781F-D43F-4D67-BDF8-463496026D57}">
   <cacheSource type="external" connectionId="2"/>
   <cacheFields count="3">
     <cacheField name="[Measures].[Total Revenue]" caption="Total Revenue" numFmtId="0" hierarchy="14" level="32767"/>
@@ -6832,7 +7960,7 @@
 </file>
 
 <file path=xl/pivotCache/pivotCacheDefinition7.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" saveData="0" refreshedBy="KOLADE" refreshedDate="46293.974194907409" backgroundQuery="1" createdVersion="8" refreshedVersion="8" minRefreshableVersion="3" recordCount="0" supportSubquery="1" supportAdvancedDrill="1" xr:uid="{AB4C98AA-5B9E-4439-9BC6-128A91CA7E9B}">
+<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" saveData="0" refreshedBy="KOLADE" refreshedDate="46294.664681249997" backgroundQuery="1" createdVersion="8" refreshedVersion="8" minRefreshableVersion="3" recordCount="0" supportSubquery="1" supportAdvancedDrill="1" xr:uid="{AB4C98AA-5B9E-4439-9BC6-128A91CA7E9B}">
   <cacheSource type="external" connectionId="2"/>
   <cacheFields count="4">
     <cacheField name="[Measures].[Total Revenue]" caption="Total Revenue" numFmtId="0" hierarchy="14" level="32767"/>
@@ -6956,7 +8084,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{6064FA6F-7944-452B-AE31-2780676AB6FE}" name="PivotTable5" cacheId="4" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="10" rowHeaderCaption="Customer Type">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{6064FA6F-7944-452B-AE31-2780676AB6FE}" name="PivotTable5" cacheId="463" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="11" rowHeaderCaption="Customer Type">
   <location ref="E16:F19" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="3">
     <pivotField dataField="1" subtotalTop="0" showAll="0" defaultSubtotal="0"/>
@@ -6998,7 +8126,7 @@
     <dataField fld="0" subtotal="count" baseField="0" baseItem="0" numFmtId="164"/>
   </dataFields>
   <formats count="1">
-    <format dxfId="0">
+    <format dxfId="81">
       <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
     </format>
   </formats>
@@ -7080,7 +8208,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable2.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{0AF100AA-DF1A-4D71-811B-3645449A1C44}" name="PivotTable4" cacheId="3" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="20" rowHeaderCaption="Product Category">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{0AF100AA-DF1A-4D71-811B-3645449A1C44}" name="PivotTable4" cacheId="460" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="21" rowHeaderCaption="Product Category">
   <location ref="H3:J10" firstHeaderRow="0" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="4">
     <pivotField dataField="1" subtotalTop="0" showAll="0" defaultSubtotal="0"/>
@@ -7139,10 +8267,10 @@
     <dataField fld="2" subtotal="count" baseField="0" baseItem="0" numFmtId="1"/>
   </dataFields>
   <formats count="2">
-    <format dxfId="2">
+    <format dxfId="83">
       <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
     </format>
-    <format dxfId="1">
+    <format dxfId="82">
       <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0">
         <references count="1">
           <reference field="4294967294" count="1" selected="0">
@@ -7230,7 +8358,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable3.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{64E71DBA-0C7C-4E82-9EBA-0BFD3AA6A528}" name="PivotTable3" cacheId="2" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" rowHeaderCaption="Region">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{64E71DBA-0C7C-4E82-9EBA-0BFD3AA6A528}" name="PivotTable3" cacheId="457" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="9" rowHeaderCaption="Region">
   <location ref="E7:F13" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="2">
     <pivotField dataField="1" subtotalTop="0" showAll="0" defaultSubtotal="0"/>
@@ -7274,7 +8402,7 @@
     <dataField fld="0" subtotal="count" baseField="0" baseItem="0" numFmtId="164"/>
   </dataFields>
   <formats count="1">
-    <format dxfId="3">
+    <format dxfId="84">
       <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
     </format>
   </formats>
@@ -7321,7 +8449,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable4.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{1103CBF0-F37E-4F1B-A1F9-556AB1749F7E}" name="PivotTable2" cacheId="1" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="7" rowHeaderCaption="Month">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{1103CBF0-F37E-4F1B-A1F9-556AB1749F7E}" name="PivotTable2" cacheId="454" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="8" rowHeaderCaption="Month">
   <location ref="B7:C20" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="3">
     <pivotField dataField="1" subtotalTop="0" showAll="0" defaultSubtotal="0"/>
@@ -7394,7 +8522,7 @@
     <dataField fld="0" subtotal="count" baseField="0" baseItem="0" numFmtId="164"/>
   </dataFields>
   <formats count="1">
-    <format dxfId="4">
+    <format dxfId="85">
       <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
     </format>
   </formats>
@@ -7452,7 +8580,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable5.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{B8A81E6E-25B2-410D-B909-4CCD26BDD774}" name="PivotTable7" cacheId="6" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="7" rowHeaderCaption="Sales Channel">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{B8A81E6E-25B2-410D-B909-4CCD26BDD774}" name="PivotTable7" cacheId="469" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="12" rowHeaderCaption="Sales Channel">
   <location ref="K14:L19" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="4">
     <pivotField dataField="1" subtotalTop="0" showAll="0" defaultSubtotal="0"/>
@@ -7508,12 +8636,21 @@
     <dataField fld="0" subtotal="count" baseField="0" baseItem="0" numFmtId="164"/>
   </dataFields>
   <formats count="1">
-    <format dxfId="5">
+    <format dxfId="86">
       <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
     </format>
   </formats>
-  <chartFormats count="1">
+  <chartFormats count="2">
     <chartFormat chart="6" format="4" series="1">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="1">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+    <chartFormat chart="10" format="5" series="1">
       <pivotArea type="data" outline="0" fieldPosition="0">
         <references count="1">
           <reference field="4294967294" count="1" selected="0">
@@ -7566,7 +8703,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable6.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{CEAC143D-C410-49A6-84E4-0650729ECF4A}" name="PivotTable6" cacheId="5" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="7" rowHeaderCaption="Product">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{CEAC143D-C410-49A6-84E4-0650729ECF4A}" name="PivotTable6" cacheId="466" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="8" rowHeaderCaption="Product">
   <location ref="H14:I20" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="3">
     <pivotField dataField="1" subtotalTop="0" showAll="0" defaultSubtotal="0"/>
@@ -7620,7 +8757,7 @@
     <dataField fld="0" subtotal="count" baseField="0" baseItem="0" numFmtId="164"/>
   </dataFields>
   <formats count="1">
-    <format dxfId="6">
+    <format dxfId="87">
       <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
     </format>
   </formats>
@@ -7687,7 +8824,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable7.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{73C83F22-FD42-40B0-B77F-FC29D10C6792}" name="PivotTable1" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{73C83F22-FD42-40B0-B77F-FC29D10C6792}" name="PivotTable1" cacheId="451" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
   <location ref="B3:E4" firstHeaderRow="0" firstDataRow="1" firstDataCol="0"/>
   <pivotFields count="5">
     <pivotField dataField="1" subtotalTop="0" showAll="0" defaultSubtotal="0"/>
@@ -7723,7 +8860,7 @@
     <dataField fld="3" subtotal="count" baseField="0" baseItem="0" numFmtId="164"/>
   </dataFields>
   <formats count="2">
-    <format dxfId="8">
+    <format dxfId="89">
       <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0">
         <references count="1">
           <reference field="4294967294" count="1" selected="0">
@@ -7732,7 +8869,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="7">
+    <format dxfId="88">
       <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0">
         <references count="1">
           <reference field="4294967294" count="1" selected="0">
@@ -7823,6 +8960,7 @@
 <slicers xmlns="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" mc:Ignorable="x xr10">
   <slicer name="Region" xr10:uid="{3858884F-8DE2-4BF4-82FC-74445EAF3DAD}" cache="Slicer_Region" caption="Region" columnCount="5" level="1" style="Slicer Style 1" rowHeight="257175"/>
   <slicer name="Region 1" xr10:uid="{886D3A88-C167-4044-9C15-0BBC7B5B5AE2}" cache="Slicer_Region" caption="Region" columnCount="5" level="1" style="Slicer Style 1" rowHeight="257175"/>
+  <slicer name="Region 2" xr10:uid="{D1B61C71-D6CF-45AE-825B-EB1FC13275AF}" cache="Slicer_Region" caption="Region" columnCount="5" level="1" style="Slicer Style 1" rowHeight="257175"/>
 </slicers>
 </file>
 

</xml_diff>